<commit_message>
feat(form): 升級 Tab 3 定型化契約變數代理引擎與 A4 純淨列印 (ADAD Master Version 49)
</commit_message>
<xml_diff>
--- a/document/資料庫、資料處理/帳務.xlsx
+++ b/document/資料庫、資料處理/帳務.xlsx
@@ -627,7 +627,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>月嫂撥款 王明</t>
+          <t>月嫂撥款 高芳</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
@@ -762,7 +762,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>月嫂撥款 黃婷</t>
+          <t>月嫂撥款 李翔英</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -897,7 +897,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>月嫂撥款 劉偉安</t>
+          <t>月嫂撥款 林豪</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>月嫂撥款 高傑宇</t>
+          <t>月嫂撥款 李威</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>月嫂撥款 陳茹</t>
+          <t>月嫂撥款 林君</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>王明</t>
+          <t>高芳</t>
         </is>
       </c>
       <c r="E1" t="n">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>王明</t>
+          <t>高芳</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>黃婷</t>
+          <t>李翔英</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>黃婷</t>
+          <t>李翔英</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>劉偉安</t>
+          <t>林豪</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>劉偉安</t>
+          <t>林豪</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>高傑宇</t>
+          <t>李威</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>高傑宇</t>
+          <t>李威</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>陳茹</t>
+          <t>林君</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>陳茹</t>
+          <t>林君</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>胡明</t>
+          <t>許晴</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>胡明</t>
+          <t>許晴</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>郭翔</t>
+          <t>郭安</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>郭翔</t>
+          <t>郭安</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>周晴</t>
+          <t>王翔</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>周晴</t>
+          <t>王翔</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>賴宥</t>
+          <t>李嘉</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>賴宥</t>
+          <t>李嘉</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>黃美雅</t>
+          <t>高洋</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>黃美雅</t>
+          <t>高洋</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">

</xml_diff>

<commit_message>
feat: add MCP plan, config, and sync files
</commit_message>
<xml_diff>
--- a/document/資料庫、資料處理/帳務.xlsx
+++ b/document/資料庫、資料處理/帳務.xlsx
@@ -530,10 +530,10 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="I3" t="n">
-        <v>502000</v>
+        <v>502500</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -575,10 +575,10 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>28000</v>
+        <v>72500</v>
       </c>
       <c r="I4" t="n">
-        <v>530000</v>
+        <v>575000</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -619,15 +619,15 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>25500</v>
+        <v>63750</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>504500</v>
+        <v>511250</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>月嫂撥款 張芳</t>
+          <t>月嫂撥款 趙偉洋</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
@@ -668,7 +668,7 @@
         <v>2500</v>
       </c>
       <c r="I6" t="n">
-        <v>507000</v>
+        <v>513750</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -710,10 +710,10 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>35000</v>
+        <v>60000</v>
       </c>
       <c r="I7" t="n">
-        <v>542000</v>
+        <v>573750</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -754,15 +754,15 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>31875</v>
+        <v>53125</v>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>510125</v>
+        <v>520625</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>月嫂撥款 楊琪</t>
+          <t>月嫂撥款 劉傑廷</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -800,10 +800,10 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="I9" t="n">
-        <v>514125</v>
+        <v>523125</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -845,10 +845,10 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>26000</v>
+        <v>35000</v>
       </c>
       <c r="I10" t="n">
-        <v>540125</v>
+        <v>558125</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -889,15 +889,15 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>25500</v>
+        <v>31875</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>514625</v>
+        <v>526250</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>月嫂撥款 張涵</t>
+          <t>月嫂撥款 趙美</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -935,10 +935,10 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>4400</v>
+        <v>2200</v>
       </c>
       <c r="I12" t="n">
-        <v>519025</v>
+        <v>528450</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -980,10 +980,10 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>61600</v>
+        <v>63800</v>
       </c>
       <c r="I13" t="n">
-        <v>580625</v>
+        <v>592250</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1028,11 +1028,11 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>524525</v>
+        <v>536150</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>月嫂撥款 周雅</t>
+          <t>月嫂撥款 郭宏</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -1070,10 +1070,10 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="I15" t="n">
-        <v>527025</v>
+        <v>538150</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1115,10 +1115,10 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>35000</v>
+        <v>38000</v>
       </c>
       <c r="I16" t="n">
-        <v>562025</v>
+        <v>576150</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1159,15 +1159,15 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>31875</v>
+        <v>34000</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>530150</v>
+        <v>542150</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>月嫂撥款 張宇</t>
+          <t>月嫂撥款 楊萱君</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -1205,10 +1205,10 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="I18" t="n">
-        <v>534150</v>
+        <v>547150</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1250,10 +1250,10 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>36000</v>
+        <v>32500</v>
       </c>
       <c r="I19" t="n">
-        <v>570150</v>
+        <v>579650</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1295,10 +1295,10 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>4000</v>
+        <v>2200</v>
       </c>
       <c r="I20" t="n">
-        <v>574150</v>
+        <v>581850</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1340,10 +1340,10 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>26000</v>
+        <v>52800</v>
       </c>
       <c r="I21" t="n">
-        <v>600150</v>
+        <v>634650</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1385,10 +1385,10 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="I22" t="n">
-        <v>605150</v>
+        <v>636650</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1430,10 +1430,10 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>2000</v>
+        <v>4400</v>
       </c>
       <c r="I23" t="n">
-        <v>607150</v>
+        <v>641050</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1475,10 +1475,10 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="I24" t="n">
-        <v>609150</v>
+        <v>643550</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
         <v>2500</v>
       </c>
       <c r="I25" t="n">
-        <v>611650</v>
+        <v>646050</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1572,7 +1572,7 @@
         <v>15000</v>
       </c>
       <c r="I26" t="n">
-        <v>626650</v>
+        <v>661050</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         <v>3000</v>
       </c>
       <c r="I27" t="n">
-        <v>629650</v>
+        <v>664050</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>張芳</t>
+          <t>趙偉洋</t>
         </is>
       </c>
       <c r="E1" t="n">
@@ -1682,14 +1682,14 @@
         </is>
       </c>
       <c r="I1" t="n">
-        <v>30000</v>
+        <v>75000</v>
       </c>
       <c r="J1" t="n">
-        <v>25500</v>
+        <v>63750</v>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>張芳</t>
+          <t>趙偉洋</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>楊琪</t>
+          <t>劉傑廷</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1732,14 +1732,14 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>37500</v>
+        <v>62500</v>
       </c>
       <c r="J2" t="n">
-        <v>31875</v>
+        <v>53125</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>楊琪</t>
+          <t>劉傑廷</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>張涵</t>
+          <t>趙美</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1782,14 +1782,14 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>30000</v>
+        <v>37500</v>
       </c>
       <c r="J3" t="n">
-        <v>25500</v>
+        <v>31875</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>張涵</t>
+          <t>趙美</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>周雅</t>
+          <t>郭宏</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>周雅</t>
+          <t>郭宏</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>張宇</t>
+          <t>楊萱君</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1882,14 +1882,14 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>37500</v>
+        <v>40000</v>
       </c>
       <c r="J5" t="n">
-        <v>31875</v>
+        <v>34000</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>張宇</t>
+          <t>楊萱君</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>吳廷</t>
+          <t>楊婷強</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1932,14 +1932,14 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>40000</v>
+        <v>37500</v>
       </c>
       <c r="J6" t="n">
-        <v>34000</v>
+        <v>31875</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>吳廷</t>
+          <t>楊婷強</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>吳冠</t>
+          <t>林嘉</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1982,14 +1982,14 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>30000</v>
+        <v>55000</v>
       </c>
       <c r="J7" t="n">
-        <v>25500</v>
+        <v>46750</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>吳冠</t>
+          <t>林嘉</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>郭欣</t>
+          <t>張芳</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -2032,14 +2032,14 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>37500</v>
+        <v>50000</v>
       </c>
       <c r="J8" t="n">
-        <v>31875</v>
+        <v>42500</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>郭欣</t>
+          <t>張芳</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>陳俊英</t>
+          <t>楊俊</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -2082,14 +2082,14 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>60000</v>
+        <v>33000</v>
       </c>
       <c r="J9" t="n">
-        <v>51000</v>
+        <v>28050</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>陳俊英</t>
+          <t>楊俊</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>李強宏</t>
+          <t>吳雅明</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -2132,14 +2132,14 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>50000</v>
+        <v>62500</v>
       </c>
       <c r="J10" t="n">
-        <v>42500</v>
+        <v>53125</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>李強宏</t>
+          <t>吳雅明</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">

</xml_diff>

<commit_message>
LINE BOT MENU WEBHOOK LIFF JSON
</commit_message>
<xml_diff>
--- a/document/資料庫、資料處理/帳務.xlsx
+++ b/document/資料庫、資料處理/帳務.xlsx
@@ -627,7 +627,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>月嫂撥款 王明</t>
+          <t>月嫂撥款 郭強琪</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
@@ -762,7 +762,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>月嫂撥款 黃婷</t>
+          <t>月嫂撥款 趙雅廷</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -897,7 +897,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>月嫂撥款 劉偉安</t>
+          <t>月嫂撥款 李欣</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>月嫂撥款 高傑宇</t>
+          <t>月嫂撥款 許威</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>月嫂撥款 陳茹</t>
+          <t>月嫂撥款 劉偉</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>王明</t>
+          <t>郭強琪</t>
         </is>
       </c>
       <c r="E1" t="n">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>王明</t>
+          <t>郭強琪</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>黃婷</t>
+          <t>趙雅廷</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>黃婷</t>
+          <t>趙雅廷</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>劉偉安</t>
+          <t>李欣</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>劉偉安</t>
+          <t>李欣</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>高傑宇</t>
+          <t>許威</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>高傑宇</t>
+          <t>許威</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>陳茹</t>
+          <t>劉偉</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>陳茹</t>
+          <t>劉偉</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>胡明</t>
+          <t>趙洋</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>胡明</t>
+          <t>趙洋</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>郭翔</t>
+          <t>吳欣</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>郭翔</t>
+          <t>吳欣</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>周晴</t>
+          <t>許芳</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>周晴</t>
+          <t>許芳</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>賴宥</t>
+          <t>徐宇傑</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>賴宥</t>
+          <t>徐宇傑</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>黃美雅</t>
+          <t>趙強奕</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>黃美雅</t>
+          <t>趙強奕</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">

</xml_diff>

<commit_message>
Refactor labor union workflows and trim unused code
</commit_message>
<xml_diff>
--- a/document/資料庫、資料處理/帳務.xlsx
+++ b/document/資料庫、資料處理/帳務.xlsx
@@ -530,10 +530,10 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="I3" t="n">
-        <v>504000</v>
+        <v>502500</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -575,10 +575,10 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>36000</v>
+        <v>35000</v>
       </c>
       <c r="I4" t="n">
-        <v>540000</v>
+        <v>537500</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -619,15 +619,15 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>34000</v>
+        <v>31875</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>506000</v>
+        <v>505625</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>月嫂撥款 吳晴宇</t>
+          <t>月嫂撥款 蔡嘉</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
@@ -668,7 +668,7 @@
         <v>2500</v>
       </c>
       <c r="I6" t="n">
-        <v>508500</v>
+        <v>508125</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -710,10 +710,10 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>35000</v>
+        <v>72500</v>
       </c>
       <c r="I7" t="n">
-        <v>543500</v>
+        <v>580625</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -754,15 +754,15 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>31875</v>
+        <v>63750</v>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>511625</v>
+        <v>516875</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>月嫂撥款 劉芳偉</t>
+          <t>月嫂撥款 徐華</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -800,10 +800,10 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="I9" t="n">
-        <v>515625</v>
+        <v>519375</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -845,10 +845,10 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>56000</v>
+        <v>47500</v>
       </c>
       <c r="I10" t="n">
-        <v>571625</v>
+        <v>566875</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -889,15 +889,15 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>51000</v>
+        <v>42500</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>520625</v>
+        <v>524375</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>月嫂撥款 林欣</t>
+          <t>月嫂撥款 張洋</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -935,10 +935,10 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="I12" t="n">
-        <v>522625</v>
+        <v>526875</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -980,10 +980,10 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>58000</v>
+        <v>72500</v>
       </c>
       <c r="I13" t="n">
-        <v>580625</v>
+        <v>599375</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1024,15 +1024,15 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>51000</v>
+        <v>63750</v>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>529625</v>
+        <v>535625</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>月嫂撥款 賴華萱</t>
+          <t>月嫂撥款 陳宥</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -1070,10 +1070,10 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>4400</v>
+        <v>2500</v>
       </c>
       <c r="I15" t="n">
-        <v>534025</v>
+        <v>538125</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1115,10 +1115,10 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>39600</v>
+        <v>35000</v>
       </c>
       <c r="I16" t="n">
-        <v>573625</v>
+        <v>573125</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1159,15 +1159,15 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>37400</v>
+        <v>31875</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>536225</v>
+        <v>541250</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>月嫂撥款 林俊美</t>
+          <t>月嫂撥款 趙冠安</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -1205,10 +1205,10 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>2200</v>
+        <v>2500</v>
       </c>
       <c r="I18" t="n">
-        <v>538425</v>
+        <v>543750</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1250,10 +1250,10 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>52800</v>
+        <v>47500</v>
       </c>
       <c r="I19" t="n">
-        <v>591225</v>
+        <v>591250</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
         <v>4400</v>
       </c>
       <c r="I20" t="n">
-        <v>595625</v>
+        <v>595650</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1340,10 +1340,10 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>61600</v>
+        <v>39600</v>
       </c>
       <c r="I21" t="n">
-        <v>657225</v>
+        <v>635250</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1385,10 +1385,10 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="I22" t="n">
-        <v>661225</v>
+        <v>640250</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1430,10 +1430,10 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>2500</v>
+        <v>2200</v>
       </c>
       <c r="I23" t="n">
-        <v>663725</v>
+        <v>642450</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1475,10 +1475,10 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>4400</v>
+        <v>4000</v>
       </c>
       <c r="I24" t="n">
-        <v>668125</v>
+        <v>646450</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
         <v>2500</v>
       </c>
       <c r="I25" t="n">
-        <v>670625</v>
+        <v>648950</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1572,7 +1572,7 @@
         <v>15000</v>
       </c>
       <c r="I26" t="n">
-        <v>685625</v>
+        <v>663950</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         <v>3000</v>
       </c>
       <c r="I27" t="n">
-        <v>688625</v>
+        <v>666950</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>吳晴宇</t>
+          <t>蔡嘉</t>
         </is>
       </c>
       <c r="E1" t="n">
@@ -1682,14 +1682,14 @@
         </is>
       </c>
       <c r="I1" t="n">
-        <v>40000</v>
+        <v>37500</v>
       </c>
       <c r="J1" t="n">
-        <v>34000</v>
+        <v>31875</v>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>吳晴宇</t>
+          <t>蔡嘉</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>劉芳偉</t>
+          <t>徐華</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1732,14 +1732,14 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>37500</v>
+        <v>75000</v>
       </c>
       <c r="J2" t="n">
-        <v>31875</v>
+        <v>63750</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>劉芳偉</t>
+          <t>徐華</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>林欣</t>
+          <t>張洋</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1782,14 +1782,14 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="J3" t="n">
-        <v>51000</v>
+        <v>42500</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>林欣</t>
+          <t>張洋</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>賴華萱</t>
+          <t>陳宥</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1832,14 +1832,14 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>60000</v>
+        <v>75000</v>
       </c>
       <c r="J4" t="n">
-        <v>51000</v>
+        <v>63750</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>賴華萱</t>
+          <t>陳宥</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>林俊美</t>
+          <t>趙冠安</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1882,14 +1882,14 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>44000</v>
+        <v>37500</v>
       </c>
       <c r="J5" t="n">
-        <v>37400</v>
+        <v>31875</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>林俊美</t>
+          <t>趙冠安</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>林強</t>
+          <t>張雅宏</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1932,14 +1932,14 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>55000</v>
+        <v>50000</v>
       </c>
       <c r="J6" t="n">
-        <v>46750</v>
+        <v>42500</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>林強</t>
+          <t>張雅宏</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>蔡雅</t>
+          <t>賴嘉</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1982,14 +1982,14 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>66000</v>
+        <v>44000</v>
       </c>
       <c r="J7" t="n">
-        <v>56100</v>
+        <v>37400</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>蔡雅</t>
+          <t>賴嘉</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>賴晴</t>
+          <t>劉豪涵</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -2032,14 +2032,14 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="J8" t="n">
-        <v>34000</v>
+        <v>42500</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>賴晴</t>
+          <t>劉豪涵</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>吳明強</t>
+          <t>楊茹強</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -2082,14 +2082,14 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>75000</v>
+        <v>44000</v>
       </c>
       <c r="J9" t="n">
-        <v>63750</v>
+        <v>37400</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>吳明強</t>
+          <t>楊茹強</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>李安俊</t>
+          <t>李嘉</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -2132,14 +2132,14 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>44000</v>
+        <v>60000</v>
       </c>
       <c r="J10" t="n">
-        <v>37400</v>
+        <v>51000</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>李安俊</t>
+          <t>李嘉</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">

</xml_diff>